<commit_message>
by passing the certificate error message
</commit_message>
<xml_diff>
--- a/reports/weather_report.xlsx
+++ b/reports/weather_report.xlsx
@@ -468,10 +468,10 @@
         <v>46269</v>
       </c>
       <c r="C3" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="D3" t="n">
-        <v>2.1</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="4">
@@ -484,10 +484,10 @@
         <v>46270</v>
       </c>
       <c r="C4" t="n">
-        <v>21</v>
+        <v>21.2</v>
       </c>
       <c r="D4" t="n">
-        <v>0.25</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="5">
@@ -788,7 +788,7 @@
         <v>46268</v>
       </c>
       <c r="C23" t="n">
-        <v>24.7</v>
+        <v>25.3</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -804,10 +804,10 @@
         <v>46269</v>
       </c>
       <c r="C24" t="n">
-        <v>21.2</v>
+        <v>21.4</v>
       </c>
       <c r="D24" t="n">
-        <v>1.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="25">
@@ -820,7 +820,7 @@
         <v>46270</v>
       </c>
       <c r="C25" t="n">
-        <v>21.2</v>
+        <v>22.3</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -1236,7 +1236,7 @@
         <v>46268</v>
       </c>
       <c r="C51" t="n">
-        <v>27.2</v>
+        <v>27.7</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
@@ -1252,7 +1252,7 @@
         <v>46269</v>
       </c>
       <c r="C52" t="n">
-        <v>27.2</v>
+        <v>27.5</v>
       </c>
       <c r="D52" t="n">
         <v>0</v>

</xml_diff>